<commit_message>
docs(examples): rewrite charts.sh master showcase + tables.sh pptx to high-level API
charts.sh / charts.py: the 8-chart master showcase now builds via the high-level
`add --type chart` command (chartType + cell dataRange or inline data + styling:
combo secondary axis, 3D view, scatter trendline, exploded 3D pie, stock OHLC
up/down bars, filled radar, multi-ring doughnut) instead of hand-authored chart
XML. Only Chart 5 (bubble) stays on raw-set — the high-level command can't map a
dataRange to a single x/y/size series. charts.md rewritten from a TODO stub into
an annotated guide. (The redundant charts/charts-demo four-set was already
removed; README now points to the charts/ per-type subdirectory.)

tables.sh: the PowerPoint report's title and data-table slides now use
`add slide/shape/table` + `set background` + per-cell `set` instead of raw-set
replacing the whole /p:sld. Slide 3 was already high-level.
</commit_message>
<xml_diff>
--- a/examples/excel/charts.xlsx
+++ b/examples/excel/charts.xlsx
@@ -3,9 +3,9 @@
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="rId1"/>
-    <x:sheet name="Analysis" sheetId="2" r:id="Rf74baf23fd474248"/>
-    <x:sheet name="StockData" sheetId="3" r:id="Rdc6db63004734218"/>
-    <x:sheet name="Assessment" sheetId="4" r:id="R4d25e253b6004d63"/>
+    <x:sheet name="Analysis" sheetId="2" r:id="Rd13be34a91054376"/>
+    <x:sheet name="StockData" sheetId="3" r:id="R4099f931d8e64710"/>
+    <x:sheet name="Assessment" sheetId="4" r:id="R81ea73abbd08410c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -225,24 +225,14 @@
     <c:title>
       <c:tx>
         <c:rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1600" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="1F4E79"/>
-                </a:solidFill>
-                <a:latin typeface="Microsoft YaHei"/>
-                <a:ea typeface="Microsoft YaHei"/>
-              </a:defRPr>
+              <a:defRPr sz="1400" b="1"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1600" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="1F4E79"/>
-                </a:solidFill>
-              </a:rPr>
+              <a:rPr lang="en-US" sz="1400" b="1"/>
               <a:t>Monthly Sales and YoY Growth Trend</a:t>
             </a:r>
           </a:p>
@@ -260,41 +250,100 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$B$1</c:f>
-            </c:strRef>
+            <c:v>East Sales</c:v>
           </c:tx>
           <c:spPr>
-            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:srgbClr val="1F4E79"/>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:srgbClr val="2E75B6"/>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000"/>
-            </a:gradFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="35000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="2E75B6"/>
+            </a:solidFill>
           </c:spPr>
           <c:cat>
             <c:strRef>
               <c:f>Sheet1!$A$2:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Sheet1!$B$2:$B$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>135</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>148</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>162</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>155</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>178</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>210</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>188</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>172</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>165</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>198</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -302,41 +351,100 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$C$1</c:f>
-            </c:strRef>
+            <c:v>South Sales</c:v>
           </c:tx>
           <c:spPr>
-            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:srgbClr val="C55A11"/>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:srgbClr val="ED7D31"/>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000"/>
-            </a:gradFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="35000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="9DC3E6"/>
+            </a:solidFill>
           </c:spPr>
           <c:cat>
             <c:strRef>
               <c:f>Sheet1!$A$2:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Sheet1!$C$2:$C$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>108</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>115</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>128</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>142</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>155</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>168</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>175</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>160</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>148</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>135</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>158</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -344,41 +452,201 @@
           <c:idx val="2"/>
           <c:order val="2"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$D$1</c:f>
-            </c:strRef>
+            <c:v>North Sales</c:v>
           </c:tx>
           <c:spPr>
-            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rotWithShape="1">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:srgbClr val="548235"/>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:srgbClr val="70AD47"/>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000"/>
-            </a:gradFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="35000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="BDD7EE"/>
+            </a:solidFill>
           </c:spPr>
           <c:cat>
             <c:strRef>
               <c:f>Sheet1!$A$2:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Sheet1!$D$2:$D$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>88</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>92</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>105</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>118</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>125</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>138</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>145</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>152</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>122</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>142</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:v>Total</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="C55A11"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$2:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$E$2:$E$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>303</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>335</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>368</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>408</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>422</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>471</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>508</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>537</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>488</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>450</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>422</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>498</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -389,79 +657,110 @@
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="3"/>
-          <c:order val="3"/>
+          <c:idx val="4"/>
+          <c:order val="4"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$F$1</c:f>
-            </c:strRef>
+            <c:v>YoY Growth %</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="38100" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
                 <a:srgbClr val="FF0000"/>
               </a:solidFill>
-              <a:prstDash val="solid"/>
-              <a:round/>
             </a:ln>
           </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="8"/>
-            <c:spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:ln>
-            </c:spPr>
-          </c:marker>
-          <c:dLbls>
-            <c:numFmt formatCode="0.0&quot;%&quot;" sourceLinked="0"/>
-            <c:spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:noFill/>
-              </a:ln>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr sz="900" b="1">
-                    <a:solidFill>
-                      <a:srgbClr val="FF0000"/>
-                    </a:solidFill>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>Sheet1!$A$2:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Sheet1!$F$2:$F$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>5.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>12.3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>15.6</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10.2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>18.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>22.1</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>25.3</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>16.8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>11.2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>7.5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>19.8</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
-          <c:smooth val="1"/>
         </c:ser>
-        <c:marker val="1"/>
-        <c:axId val="1"/>
         <c:axId val="3"/>
+        <c:axId val="4"/>
       </c:lineChart>
       <c:catAx>
         <c:axId val="1"/>
@@ -470,28 +769,14 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-            <a:solidFill>
-              <a:srgbClr val="BFBFBF"/>
-            </a:solidFill>
-          </a:ln>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr sz="1000">
-                <a:solidFill>
-                  <a:srgbClr val="404040"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
         <c:crossAx val="2"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="2"/>
@@ -500,98 +785,68 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
+        <c:majorGridlines/>
         <c:title>
           <c:tx>
             <c:rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
               <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
               <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
-                  <a:defRPr sz="1000">
-                    <a:solidFill>
-                      <a:srgbClr val="404040"/>
-                    </a:solidFill>
-                  </a:defRPr>
+                  <a:defRPr sz="1400" b="1"/>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US" sz="1000"/>
+                  <a:rPr lang="en-US" sz="1400" b="1"/>
                   <a:t>Sales (10K)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
           </c:tx>
+          <c:overlay val="0"/>
         </c:title>
-        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
-        <c:spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-            <a:solidFill>
-              <a:srgbClr val="BFBFBF"/>
-            </a:solidFill>
-          </a:ln>
-        </c:spPr>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
         <c:crossAx val="1"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
       </c:valAx>
+      <c:catAx>
+        <c:axId val="3"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="none"/>
+        <c:crossAx val="4"/>
+        <c:crosses val="autoZero"/>
+      </c:catAx>
       <c:valAx>
-        <c:axId val="3"/>
+        <c:axId val="4"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="r"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr sz="1000">
-                    <a:solidFill>
-                      <a:srgbClr val="FF0000"/>
-                    </a:solidFill>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US" sz="1000"/>
-                  <a:t>YoY Growth (%)</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-        </c:title>
-        <c:numFmt formatCode="0.0&quot;%&quot;" sourceLinked="0"/>
-        <c:spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-            <a:solidFill>
-              <a:srgbClr val="FF0000">
-                <a:alpha val="50000"/>
-              </a:srgbClr>
-            </a:solidFill>
-          </a:ln>
-        </c:spPr>
-        <c:crossAx val="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="3"/>
         <c:crosses val="max"/>
+        <c:crossBetween val="between"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
       <c:overlay val="0"/>
-      <c:txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr>
-            <a:defRPr sz="1000">
-              <a:solidFill>
-                <a:srgbClr val="404040"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
     </c:legend>
     <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
   </c:chart>
 </c:chartSpace>
 </file>
@@ -606,14 +861,10 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1600" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="1F4E79"/>
-                </a:solidFill>
-              </a:defRPr>
+              <a:defRPr sz="1400" b="1"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1600" b="1"/>
+              <a:rPr lang="en-US" sz="1400" b="1"/>
               <a:t>3D Regional Sales Comparison</a:t>
             </a:r>
           </a:p>
@@ -624,8 +875,6 @@
     <c:view3D>
       <c:rotX val="15"/>
       <c:rotY val="20"/>
-      <c:depthPercent val="100"/>
-      <c:rAngAx val="1"/>
       <c:perspective val="30"/>
     </c:view3D>
     <c:plotArea>
@@ -638,34 +887,100 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$B$1</c:f>
-            </c:strRef>
+            <c:v>East Sales</c:v>
           </c:tx>
           <c:spPr>
-            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:srgbClr val="4472C4"/>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:srgbClr val="5B9BD5"/>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:srgbClr val="9DC3E6"/>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000"/>
-            </a:gradFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="4472C4"/>
+            </a:solidFill>
           </c:spPr>
           <c:cat>
             <c:strRef>
               <c:f>Sheet1!$A$2:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Sheet1!$B$2:$B$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>135</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>148</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>162</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>155</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>178</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>210</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>188</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>172</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>165</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>198</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -673,34 +988,100 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$C$1</c:f>
-            </c:strRef>
+            <c:v>South Sales</c:v>
           </c:tx>
           <c:spPr>
-            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:srgbClr val="ED7D31"/>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:srgbClr val="F4B183"/>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:srgbClr val="F8CBAD"/>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000"/>
-            </a:gradFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="ED7D31"/>
+            </a:solidFill>
           </c:spPr>
           <c:cat>
             <c:strRef>
               <c:f>Sheet1!$A$2:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Sheet1!$C$2:$C$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>108</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>115</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>128</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>142</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>155</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>168</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>175</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>160</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>148</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>135</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>158</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -708,69 +1089,148 @@
           <c:idx val="2"/>
           <c:order val="2"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$D$1</c:f>
-            </c:strRef>
+            <c:v>North Sales</c:v>
           </c:tx>
           <c:spPr>
-            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:gsLst>
-                <a:gs pos="0">
-                  <a:srgbClr val="70AD47"/>
-                </a:gs>
-                <a:gs pos="50000">
-                  <a:srgbClr val="A9D18E"/>
-                </a:gs>
-                <a:gs pos="100000">
-                  <a:srgbClr val="C5E0B4"/>
-                </a:gs>
-              </a:gsLst>
-              <a:lin ang="5400000"/>
-            </a:gradFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="70AD47"/>
+            </a:solidFill>
           </c:spPr>
           <c:cat>
             <c:strRef>
               <c:f>Sheet1!$A$2:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Sheet1!$D$2:$D$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>88</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>92</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>105</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>118</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>125</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>138</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>145</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>152</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>122</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>142</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:shape val="cylinder"/>
-        <c:axId val="10"/>
-        <c:axId val="20"/>
-        <c:axId val="30"/>
+        <c:gapWidth val="150"/>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+        <c:axId val="3"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="10"/>
+        <c:axId val="1"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:crossAx val="20"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="2"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="20"/>
+        <c:axId val="2"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
-        <c:crossAx val="10"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
       </c:valAx>
       <c:serAx>
-        <c:axId val="30"/>
+        <c:axId val="3"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:crossAx val="20"/>
+        <c:crossAx val="2"/>
       </c:serAx>
     </c:plotArea>
     <c:legend>
@@ -778,6 +1238,7 @@
       <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
   </c:chart>
 </c:chartSpace>
 </file>
@@ -792,14 +1253,10 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1600" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="7030A0"/>
-                </a:solidFill>
-              </a:defRPr>
+              <a:defRPr sz="1400" b="1"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1600" b="1"/>
+              <a:rPr lang="en-US" sz="1400" b="1"/>
               <a:t>Ad Spend vs Sales Correlation</a:t>
             </a:r>
           </a:p>
@@ -816,74 +1273,138 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Analysis!$B$1</c:f>
-            </c:strRef>
+            <c:v>Sales (10K)</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
-              <a:noFill/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
+              <a:solidFill>
+                <a:srgbClr val="7030A0"/>
+              </a:solidFill>
             </a:ln>
           </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="10"/>
-            <c:spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="7030A0">
-                  <a:alpha val="70000"/>
-                </a:srgbClr>
-              </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
-                <a:solidFill>
-                  <a:srgbClr val="7030A0"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:outerShdw blurRad="40000" dist="20000" dir="5400000">
-                  <a:srgbClr val="000000">
-                    <a:alpha val="30000"/>
-                  </a:srgbClr>
-                </a:outerShdw>
-              </a:effectLst>
-            </c:spPr>
-          </c:marker>
           <c:trendline>
-            <c:spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400" cap="rnd">
-                <a:solidFill>
-                  <a:srgbClr val="FF0000"/>
-                </a:solidFill>
-                <a:prstDash val="dash"/>
-                <a:round/>
-              </a:ln>
-            </c:spPr>
             <c:trendlineType val="linear"/>
-            <c:dispRSqr val="1"/>
-            <c:dispEq val="1"/>
           </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>Analysis!$A$2:$A$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>58</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>65</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>72</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>88</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>105</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>115</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
               <c:f>Analysis!$B$2:$B$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>68</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>155</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>220</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>290</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>335</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>370</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>410</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>445</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>550</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="100"/>
-        <c:axId val="200"/>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="100"/>
+        <c:axId val="1"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:majorGridlines/>
         <c:title>
           <c:tx>
             <c:rich>
@@ -891,59 +1412,40 @@
               <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
               <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
-                  <a:defRPr sz="1000"/>
+                  <a:defRPr sz="1400" b="1"/>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US" sz="1000"/>
-                  <a:t>Ad Spend (10K)</a:t>
+                  <a:rPr lang="en-US" sz="1400" b="1"/>
+                  <a:t>Sales (10K)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
           </c:tx>
+          <c:overlay val="0"/>
         </c:title>
-        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
-        <c:spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-            <a:solidFill>
-              <a:srgbClr val="BFBFBF"/>
-            </a:solidFill>
-          </a:ln>
-        </c:spPr>
-        <c:crossAx val="200"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="2"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="200"/>
+        <c:axId val="2"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr sz="1000"/>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US" sz="1000"/>
-                  <a:t>Sales (10K)</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-        </c:title>
-        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
-        <c:spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-            <a:solidFill>
-              <a:srgbClr val="BFBFBF"/>
-            </a:solidFill>
-          </a:ln>
-        </c:spPr>
-        <c:crossAx val="100"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -951,6 +1453,7 @@
       <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
   </c:chart>
 </c:chartSpace>
 </file>
@@ -965,15 +1468,11 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1600" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="1F4E79"/>
-                </a:solidFill>
-              </a:defRPr>
+              <a:defRPr sz="1400" b="1"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1600" b="1"/>
-              <a:t>Annual Regional Sales Share (3D)</a:t>
+              <a:rPr lang="en-US" sz="1400" b="1"/>
+              <a:t>July Regional Sales Share (3D)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -983,7 +1482,6 @@
     <c:view3D>
       <c:rotX val="30"/>
       <c:rotY val="70"/>
-      <c:rAngAx val="0"/>
       <c:perspective val="30"/>
     </c:view3D>
     <c:plotArea>
@@ -993,121 +1491,79 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:v>Jul</c:v>
+          </c:tx>
           <c:explosion val="10"/>
           <c:dPt>
             <c:idx val="0"/>
             <c:spPr>
-              <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:gsLst>
-                  <a:gs pos="0">
-                    <a:srgbClr val="1F4E79"/>
-                  </a:gs>
-                  <a:gs pos="100000">
-                    <a:srgbClr val="4472C4"/>
-                  </a:gs>
-                </a:gsLst>
-                <a:lin ang="5400000"/>
-              </a:gradFill>
-              <a:effectLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:outerShdw blurRad="50800" dist="38100" dir="5400000">
-                  <a:srgbClr val="000000">
-                    <a:alpha val="40000"/>
-                  </a:srgbClr>
-                </a:outerShdw>
-              </a:effectLst>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="1F4E79"/>
+              </a:solidFill>
             </c:spPr>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
             <c:spPr>
-              <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:gsLst>
-                  <a:gs pos="0">
-                    <a:srgbClr val="C55A11"/>
-                  </a:gs>
-                  <a:gs pos="100000">
-                    <a:srgbClr val="ED7D31"/>
-                  </a:gs>
-                </a:gsLst>
-                <a:lin ang="5400000"/>
-              </a:gradFill>
-              <a:effectLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:outerShdw blurRad="50800" dist="38100" dir="5400000">
-                  <a:srgbClr val="000000">
-                    <a:alpha val="40000"/>
-                  </a:srgbClr>
-                </a:outerShdw>
-              </a:effectLst>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="C55A11"/>
+              </a:solidFill>
             </c:spPr>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
             <c:spPr>
-              <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:gsLst>
-                  <a:gs pos="0">
-                    <a:srgbClr val="548235"/>
-                  </a:gs>
-                  <a:gs pos="100000">
-                    <a:srgbClr val="70AD47"/>
-                  </a:gs>
-                </a:gsLst>
-                <a:lin ang="5400000"/>
-              </a:gradFill>
-              <a:effectLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:outerShdw blurRad="50800" dist="38100" dir="5400000">
-                  <a:srgbClr val="000000">
-                    <a:alpha val="40000"/>
-                  </a:srgbClr>
-                </a:outerShdw>
-              </a:effectLst>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="548235"/>
+              </a:solidFill>
             </c:spPr>
           </c:dPt>
-          <c:dLbls>
-            <c:numFmt formatCode="0.0&quot;%&quot;" sourceLinked="0"/>
-            <c:spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:noFill/>
-              </a:ln>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr sz="1100" b="1">
-                    <a:solidFill>
-                      <a:srgbClr val="FFFFFF"/>
-                    </a:solidFill>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
-            <c:showCatName val="1"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="1"/>
-          </c:dLbls>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$B$1:$D$1</c:f>
-            </c:strRef>
+            <c:strLit>
+              <c:ptCount val="3"/>
+              <c:pt idx="0">
+                <c:v>East Sales</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>South Sales</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>North Sales</c:v>
+              </c:pt>
+            </c:strLit>
           </c:cat>
           <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$B$8:$D$8</c:f>
-            </c:numRef>
+            <c:numLit>
+              <c:formatCode>General</c:formatCode>
+              <c:ptCount val="3"/>
+              <c:pt idx="0">
+                <c:v>195</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>168</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>145</c:v>
+              </c:pt>
+            </c:numLit>
           </c:val>
         </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+        </c:dLbls>
       </c:pie3DChart>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
       <c:overlay val="0"/>
     </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
   </c:chart>
 </c:chartSpace>
 </file>
@@ -1160,13 +1616,6 @@
                 <a:srgbClr val="7030A0"/>
               </a:solidFill>
             </a:ln>
-            <a:effectLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:outerShdw blurRad="40000" dist="23000" dir="5400000">
-                <a:srgbClr val="000000">
-                  <a:alpha val="25000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
           </c:spPr>
           <c:xVal>
             <c:numRef>
@@ -1262,14 +1711,10 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1600" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="C00000"/>
-                </a:solidFill>
-              </a:defRPr>
+              <a:defRPr sz="1400" b="1"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1600" b="1"/>
+              <a:rPr lang="en-US" sz="1400" b="1"/>
               <a:t>Stock Candlestick Chart (OHLC)</a:t>
             </a:r>
           </a:p>
@@ -1284,12 +1729,10 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:strRef>
-              <c:f>StockData!$B$1</c:f>
-            </c:strRef>
+            <c:v>Open</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
             </a:ln>
           </c:spPr>
@@ -1299,11 +1742,138 @@
           <c:cat>
             <c:strRef>
               <c:f>StockData!$A$2:$A$21</c:f>
+              <c:strCache>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>3/1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3/2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3/3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3/4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3/5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3/6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3/7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3/8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3/9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3/10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>3/11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>3/12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>3/13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>3/14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3/15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>3/16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>3/17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>3/18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>3/19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>3/20</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>StockData!$B$2:$B$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>52.3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>53.1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>52.8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>54.2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>55.1</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>54.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>56.2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>57.8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>58.5</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>57.2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>56.8</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>58.3</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>59.5</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>60.2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>59.8</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>61.5</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>62.3</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>61.8</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>63.5</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>64.2</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -1311,12 +1881,10 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:strRef>
-              <c:f>StockData!$C$1</c:f>
-            </c:strRef>
+            <c:v>High</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
             </a:ln>
           </c:spPr>
@@ -1326,11 +1894,138 @@
           <c:cat>
             <c:strRef>
               <c:f>StockData!$A$2:$A$21</c:f>
+              <c:strCache>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>3/1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3/2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3/3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3/4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3/5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3/6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3/7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3/8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3/9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3/10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>3/11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>3/12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>3/13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>3/14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3/15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>3/16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>3/17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>3/18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>3/19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>3/20</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>StockData!$C$2:$C$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>53.8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>54.2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>54.5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>55.8</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>56.3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>56.8</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>58.1</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>59.2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>59.8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>58.5</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>58.2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>59.8</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>61.2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>61.5</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>61.8</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>63.2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>63.8</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>63.5</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>65.2</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>65.8</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -1338,12 +2033,10 @@
           <c:idx val="2"/>
           <c:order val="2"/>
           <c:tx>
-            <c:strRef>
-              <c:f>StockData!$D$1</c:f>
-            </c:strRef>
+            <c:v>Low</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
             </a:ln>
           </c:spPr>
@@ -1353,11 +2046,138 @@
           <c:cat>
             <c:strRef>
               <c:f>StockData!$A$2:$A$21</c:f>
+              <c:strCache>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>3/1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3/2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3/3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3/4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3/5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3/6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3/7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3/8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3/9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3/10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>3/11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>3/12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>3/13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>3/14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3/15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>3/16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>3/17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>3/18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>3/19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>3/20</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>StockData!$D$2:$D$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>51.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>52.2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>51.8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>53.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>54.2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>53.8</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>55.5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>56.8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>57.2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>56.1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>55.8</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>57.5</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>58.8</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>59.2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>58.5</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>60.8</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>61.2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>60.5</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>62.8</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>63.5</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -1365,12 +2185,10 @@
           <c:idx val="3"/>
           <c:order val="3"/>
           <c:tx>
-            <c:strRef>
-              <c:f>StockData!$E$1</c:f>
-            </c:strRef>
+            <c:v>Close</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
             </a:ln>
           </c:spPr>
@@ -1380,81 +2198,193 @@
           <c:cat>
             <c:strRef>
               <c:f>StockData!$A$2:$A$21</c:f>
+              <c:strCache>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>3/1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3/2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3/3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3/4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3/5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3/6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3/7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3/8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3/9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3/10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>3/11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>3/12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>3/13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>3/14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3/15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>3/16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>3/17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>3/18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>3/19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>3/20</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>StockData!$E$2:$E$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>53.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>52.8</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>54.2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>55.1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>54.5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>56.2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>57.8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>58.5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>57.2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>56.8</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>58.3</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>59.5</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>60.2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>59.8</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>61.5</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>62.3</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>61.8</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>63.5</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>64.2</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>65.1</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:hiLowLines>
-          <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="404040"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-        </c:hiLowLines>
+        <c:hiLowLines/>
         <c:upDownBars>
-          <c:gapWidth val="100"/>
+          <c:gapWidth val="150"/>
           <c:upBars>
             <c:spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="FF0000"/>
+                <a:srgbClr val="4CAF50"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-                <a:solidFill>
-                  <a:srgbClr val="C00000"/>
-                </a:solidFill>
-              </a:ln>
             </c:spPr>
           </c:upBars>
           <c:downBars>
             <c:spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="00B050"/>
+                <a:srgbClr val="F44336"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-                <a:solidFill>
-                  <a:srgbClr val="006400"/>
-                </a:solidFill>
-              </a:ln>
             </c:spPr>
           </c:downBars>
         </c:upDownBars>
-        <c:axId val="500"/>
-        <c:axId val="600"/>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
       </c:stockChart>
       <c:catAx>
-        <c:axId val="500"/>
+        <c:axId val="1"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr sz="800"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="600"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="2"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="600"/>
+        <c:axId val="2"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:numFmt formatCode="0.00" sourceLinked="0"/>
-        <c:crossAx val="500"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1462,6 +2392,7 @@
       <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
   </c:chart>
 </c:chartSpace>
 </file>
@@ -1476,14 +2407,10 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1600" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="002060"/>
-                </a:solidFill>
-              </a:defRPr>
+              <a:defRPr sz="1400" b="1"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1600" b="1"/>
+              <a:rPr lang="en-US" sz="1400" b="1"/>
               <a:t>Product Capability Radar Comparison</a:t>
             </a:r>
           </a:p>
@@ -1500,17 +2427,10 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Assessment!$B$1</c:f>
-            </c:strRef>
+            <c:v>Product A</c:v>
           </c:tx>
           <c:spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="4472C4">
-                <a:alpha val="40000"/>
-              </a:srgbClr>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
                 <a:srgbClr val="4472C4"/>
               </a:solidFill>
@@ -1519,11 +2439,66 @@
           <c:cat>
             <c:strRef>
               <c:f>Assessment!$A$2:$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Performance</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Stability</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Usability</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Security</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Scalability</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Value</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Ecosystem</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Docs</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Assessment!$B$2:$B$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>92</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>88</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>82</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>78</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -1531,17 +2506,10 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Assessment!$C$1</c:f>
-            </c:strRef>
+            <c:v>Product B</c:v>
           </c:tx>
           <c:spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="00B050">
-                <a:alpha val="40000"/>
-              </a:srgbClr>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
                 <a:srgbClr val="00B050"/>
               </a:solidFill>
@@ -1550,11 +2518,66 @@
           <c:cat>
             <c:strRef>
               <c:f>Assessment!$A$2:$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Performance</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Stability</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Usability</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Security</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Scalability</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Value</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Ecosystem</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Docs</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Assessment!$C$2:$C$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>78</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>92</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>88</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>72</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>82</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -1562,17 +2585,10 @@
           <c:idx val="2"/>
           <c:order val="2"/>
           <c:tx>
-            <c:strRef>
-              <c:f>Assessment!$D$1</c:f>
-            </c:strRef>
+            <c:v>Product C</c:v>
           </c:tx>
           <c:spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="FFC000">
-                <a:alpha val="40000"/>
-              </a:srgbClr>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
               <a:solidFill>
                 <a:srgbClr val="FFC000"/>
               </a:solidFill>
@@ -1581,42 +2597,111 @@
           <c:cat>
             <c:strRef>
               <c:f>Assessment!$A$2:$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Performance</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Stability</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Usability</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Security</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Scalability</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Value</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Ecosystem</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Docs</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Assessment!$D$2:$D$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>76</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>92</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>72</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>78</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>92</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>88</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>70</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="700"/>
-        <c:axId val="800"/>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
       </c:radarChart>
       <c:catAx>
-        <c:axId val="700"/>
+        <c:axId val="1"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:crossAx val="800"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="2"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="800"/>
+        <c:axId val="2"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="100"/>
-          <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:crossAx val="700"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
       <c:overlay val="0"/>
     </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
   </c:chart>
 </c:chartSpace>
 </file>
@@ -1631,15 +2716,11 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1600" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="1F4E79"/>
-                </a:solidFill>
-              </a:defRPr>
+              <a:defRPr sz="1400" b="1"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1600" b="1"/>
-              <a:t>Q3 vs Q4 Regional Sales Multi-Ring</a:t>
+              <a:rPr lang="en-US" sz="1400" b="1"/>
+              <a:t>Aug vs Dec Regional Sales Multi-Ring</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1654,7 +2735,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Q3</c:v>
+            <c:v>Aug</c:v>
           </c:tx>
           <c:dPt>
             <c:idx val="0"/>
@@ -1680,56 +2761,47 @@
               </a:solidFill>
             </c:spPr>
           </c:dPt>
-          <c:dLbls>
-            <c:numFmt formatCode="0.0&quot;%&quot;" sourceLinked="0"/>
-            <c:spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:noFill/>
-              </a:ln>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr sz="900" b="1">
-                    <a:solidFill>
-                      <a:srgbClr val="FFFFFF"/>
-                    </a:solidFill>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="1"/>
-          </c:dLbls>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$B$1:$D$1</c:f>
-            </c:strRef>
+            <c:strLit>
+              <c:ptCount val="3"/>
+              <c:pt idx="0">
+                <c:v>East</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>South</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>North</c:v>
+              </c:pt>
+            </c:strLit>
           </c:cat>
           <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$B$9:$D$9</c:f>
-            </c:numRef>
+            <c:numLit>
+              <c:formatCode>General</c:formatCode>
+              <c:ptCount val="3"/>
+              <c:pt idx="0">
+                <c:v>210</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>175</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>152</c:v>
+              </c:pt>
+            </c:numLit>
           </c:val>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>Q4</c:v>
+            <c:v>Dec</c:v>
           </c:tx>
           <c:dPt>
             <c:idx val="0"/>
             <c:spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="4472C4"/>
+                <a:srgbClr val="1F4E79"/>
               </a:solidFill>
             </c:spPr>
           </c:dPt>
@@ -1737,7 +2809,7 @@
             <c:idx val="1"/>
             <c:spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="ED7D31"/>
+                <a:srgbClr val="C55A11"/>
               </a:solidFill>
             </c:spPr>
           </c:dPt>
@@ -1745,63 +2817,63 @@
             <c:idx val="2"/>
             <c:spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="70AD47"/>
+                <a:srgbClr val="548235"/>
               </a:solidFill>
             </c:spPr>
           </c:dPt>
-          <c:dLbls>
-            <c:numFmt formatCode="0.0&quot;%&quot;" sourceLinked="0"/>
-            <c:spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:noFill/>
-              </a:ln>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr sz="900" b="1">
-                    <a:solidFill>
-                      <a:srgbClr val="FFFFFF"/>
-                    </a:solidFill>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
-            <c:showCatName val="1"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="1"/>
-          </c:dLbls>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$B$1:$D$1</c:f>
-            </c:strRef>
+            <c:strLit>
+              <c:ptCount val="3"/>
+              <c:pt idx="0">
+                <c:v>East</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>South</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>North</c:v>
+              </c:pt>
+            </c:strLit>
           </c:cat>
           <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$B$13:$D$13</c:f>
-            </c:numRef>
+            <c:numLit>
+              <c:formatCode>General</c:formatCode>
+              <c:ptCount val="3"/>
+              <c:pt idx="0">
+                <c:v>198</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>158</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>142</c:v>
+              </c:pt>
+            </c:numLit>
           </c:val>
         </c:ser>
-        <c:holeSize val="40"/>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+        </c:dLbls>
+        <c:holeSize val="50"/>
       </c:doughnutChart>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
       <c:overlay val="0"/>
     </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
   </c:chart>
 </c:chartSpace>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
@@ -1814,9 +2886,9 @@
       <xdr:row>18</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
-    <xdr:graphicFrame macro="">
+    <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvPr id="2" name="Monthly Sales and YoY Growth Trend"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -1825,13 +2897,13 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R5f32f03e341a48f1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R098396f3395048f5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
@@ -1844,9 +2916,9 @@
       <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
-    <xdr:graphicFrame macro="">
+    <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvPr id="3" name="3D Regional Sales Comparison"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -1855,13 +2927,13 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R0fb89e79ac47438c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0a3955817b8b4280"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>19</xdr:col>
       <xdr:colOff>0</xdr:colOff>
@@ -1874,9 +2946,9 @@
       <xdr:row>18</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
-    <xdr:graphicFrame macro="">
+    <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 4"/>
+        <xdr:cNvPr id="4" name="July Regional Sales Share (3D)"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -1885,13 +2957,13 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="Rc37ea2ed1d234d65"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R451d0410638b46a8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>19</xdr:col>
       <xdr:colOff>0</xdr:colOff>
@@ -1904,9 +2976,9 @@
       <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
-    <xdr:graphicFrame macro="">
+    <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Chart 8"/>
+        <xdr:cNvPr id="5" name="Aug vs Dec Regional Sales Multi-Ring"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -1915,7 +2987,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R9b97efaab64c4fc2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R24496af6531145a5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1939,9 +3011,9 @@
       <xdr:row>18</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
-    <xdr:graphicFrame macro="">
+    <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 3"/>
+        <xdr:cNvPr id="2" name="Ad Spend vs Sales Correlation"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -1950,7 +3022,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R4f37a44f2dcb4bd4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0b9e84bc36eb426f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1980,7 +3052,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R8f38dfd91aa145ec"/>
+          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="Ra074047bc5574c87"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1991,7 +3063,7 @@
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
@@ -2004,9 +3076,9 @@
       <xdr:row>22</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
-    <xdr:graphicFrame macro="">
+    <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 6"/>
+        <xdr:cNvPr id="2" name="Stock Candlestick Chart (OHLC)"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -2015,7 +3087,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="Rfe978a6e5704422d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R72544edefb0949d5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2026,7 +3098,7 @@
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
@@ -2039,9 +3111,9 @@
       <xdr:row>20</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
-    <xdr:graphicFrame macro="">
+    <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 7"/>
+        <xdr:cNvPr id="2" name="Product Capability Radar Comparison"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -2050,7 +3122,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:p5="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" p5:id="R52fc8db431e44d06"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra5cd8a74935b48d9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2432,7 +3504,7 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R606676e2adee466a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re90e1709f8804316"/>
 </x:worksheet>
 </file>
 
@@ -2664,7 +3736,7 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccb94887c4c54494"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6049dbde0504cb4"/>
 </x:worksheet>
 </file>
 
@@ -3092,7 +4164,7 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd10e8f633b474643"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5029eb1676e348ee"/>
 </x:worksheet>
 </file>
 
@@ -3226,6 +4298,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88830dcb4140437a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Redb67385a92b40c7"/>
 </x:worksheet>
 </file>
</xml_diff>